<commit_message>
rtk: add custom_id support to test cases, update grid layout, and regenerate import template
</commit_message>
<xml_diff>
--- a/public/templates/test_case_import_template.xlsx
+++ b/public/templates/test_case_import_template.xlsx
@@ -397,135 +397,145 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:L3"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="40.83203125" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" customWidth="1"/>
-    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="15.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
     <col min="5" max="5" width="15.83203125" customWidth="1"/>
-    <col min="6" max="6" width="20.83203125" customWidth="1"/>
-    <col min="7" max="7" width="10.83203125" customWidth="1"/>
-    <col min="8" max="8" width="20.83203125" customWidth="1"/>
-    <col min="9" max="9" width="40.83203125" customWidth="1"/>
-    <col min="10" max="10" width="20.83203125" customWidth="1"/>
-    <col min="11" max="11" width="30.83203125" customWidth="1"/>
+    <col min="6" max="6" width="15.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
+    <col min="8" max="8" width="10.83203125" customWidth="1"/>
+    <col min="9" max="9" width="20.83203125" customWidth="1"/>
+    <col min="10" max="10" width="40.83203125" customWidth="1"/>
+    <col min="11" max="11" width="20.83203125" customWidth="1"/>
+    <col min="12" max="12" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
         <v>scenario</v>
       </c>
-      <c r="B1" t="str">
+      <c r="C1" t="str">
         <v>title</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>type</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>priority</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>automation_status</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>requirement_link</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>estimated_duration</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>precondition</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>steps</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>test_data</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>expected_result</v>
       </c>
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
+        <v>TC-001</v>
+      </c>
+      <c r="B2" t="str">
         <v>Login</v>
       </c>
-      <c r="B2" t="str">
+      <c r="C2" t="str">
         <v>Login dengan email terdaftar dan password yang benar</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>Positive</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>P0 - Critical</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>Manual</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v/>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>5</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
         <v>User is registered</v>
       </c>
-      <c r="I2" t="str" xml:space="preserve">
+      <c r="J2" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Open Login Page
 2. Enter email
 3. Enter valid password
 4. Click Login</v>
       </c>
-      <c r="J2" t="str">
+      <c r="K2" t="str">
         <v>email: test@example.com</v>
       </c>
-      <c r="K2" t="str">
+      <c r="L2" t="str">
         <v>Dashboard should be displayed</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">
       <c r="A3" t="str">
+        <v>TC-002</v>
+      </c>
+      <c r="B3" t="str">
         <v/>
       </c>
-      <c r="B3" t="str">
+      <c r="C3" t="str">
         <v>Login menggunakan email yang terdaftar dan password yang salah</v>
       </c>
-      <c r="C3" t="str">
+      <c r="D3" t="str">
         <v>Negative</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>P1 - High</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F3" t="str">
         <v>Manual</v>
       </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
         <v/>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>3</v>
       </c>
-      <c r="H3" t="str">
+      <c r="I3" t="str">
         <v/>
       </c>
-      <c r="I3" t="str" xml:space="preserve">
+      <c r="J3" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Open Login Page
 2. Enter valid email
 3. Enter WRONG password
 4. Click Login</v>
       </c>
-      <c r="J3" t="str">
+      <c r="K3" t="str">
         <v/>
       </c>
-      <c r="K3" t="str">
+      <c r="L3" t="str">
         <v>Error message "Invalid credentials" shown</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: support module column in test case import with auto-creation option
</commit_message>
<xml_diff>
--- a/public/templates/test_case_import_template.xlsx
+++ b/public/templates/test_case_import_template.xlsx
@@ -397,20 +397,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:M3"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
-    <col min="3" max="3" width="40.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="15.83203125" customWidth="1"/>
+    <col min="3" max="3" width="15.83203125" customWidth="1"/>
+    <col min="4" max="4" width="40.83203125" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" customWidth="1"/>
     <col min="6" max="6" width="15.83203125" customWidth="1"/>
-    <col min="7" max="7" width="20.83203125" customWidth="1"/>
-    <col min="8" max="8" width="10.83203125" customWidth="1"/>
-    <col min="9" max="9" width="20.83203125" customWidth="1"/>
-    <col min="10" max="10" width="40.83203125" customWidth="1"/>
-    <col min="11" max="11" width="20.83203125" customWidth="1"/>
-    <col min="12" max="12" width="30.83203125" customWidth="1"/>
+    <col min="7" max="7" width="15.83203125" customWidth="1"/>
+    <col min="8" max="8" width="20.83203125" customWidth="1"/>
+    <col min="9" max="9" width="10.83203125" customWidth="1"/>
+    <col min="10" max="10" width="20.83203125" customWidth="1"/>
+    <col min="11" max="11" width="40.83203125" customWidth="1"/>
+    <col min="12" max="12" width="20.83203125" customWidth="1"/>
+    <col min="13" max="13" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -418,36 +419,39 @@
         <v>id</v>
       </c>
       <c r="B1" t="str">
+        <v>module</v>
+      </c>
+      <c r="C1" t="str">
         <v>scenario</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>title</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>type</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>priority</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>automation_status</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>requirement_link</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>estimated_duration</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>precondition</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>steps</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>test_data</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>expected_result</v>
       </c>
     </row>
@@ -456,39 +460,42 @@
         <v>TC-001</v>
       </c>
       <c r="B2" t="str">
+        <v>Authentication</v>
+      </c>
+      <c r="C2" t="str">
         <v>Login</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>Login dengan email terdaftar dan password yang benar</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>Positive</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>P0 - Critical</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>Manual</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v/>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>5</v>
       </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
         <v>User is registered</v>
       </c>
-      <c r="J2" t="str" xml:space="preserve">
+      <c r="K2" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Open Login Page
 2. Enter email
 3. Enter valid password
 4. Click Login</v>
       </c>
-      <c r="K2" t="str">
+      <c r="L2" t="str">
         <v>email: test@example.com</v>
       </c>
-      <c r="L2" t="str">
+      <c r="M2" t="str">
         <v>Dashboard should be displayed</v>
       </c>
     </row>
@@ -497,45 +504,48 @@
         <v>TC-002</v>
       </c>
       <c r="B3" t="str">
+        <v>Authentication</v>
+      </c>
+      <c r="C3" t="str">
         <v/>
       </c>
-      <c r="C3" t="str">
+      <c r="D3" t="str">
         <v>Login menggunakan email yang terdaftar dan password yang salah</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>Negative</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F3" t="str">
         <v>P1 - High</v>
       </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
         <v>Manual</v>
       </c>
-      <c r="G3" t="str">
+      <c r="H3" t="str">
         <v/>
       </c>
-      <c r="H3">
+      <c r="I3">
         <v>3</v>
       </c>
-      <c r="I3" t="str">
+      <c r="J3" t="str">
         <v/>
       </c>
-      <c r="J3" t="str" xml:space="preserve">
+      <c r="K3" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Open Login Page
 2. Enter valid email
 3. Enter WRONG password
 4. Click Login</v>
       </c>
-      <c r="K3" t="str">
+      <c r="L3" t="str">
         <v/>
       </c>
-      <c r="L3" t="str">
+      <c r="M3" t="str">
         <v>Error message "Invalid credentials" shown</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>